<commit_message>
Logout erstellt und ausgewertet
</commit_message>
<xml_diff>
--- a/Testdaten/Testdaten von und für GPT-4/OpenCart-TestExecution Results_GPT-4.xlsx
+++ b/Testdaten/Testdaten von und für GPT-4/OpenCart-TestExecution Results_GPT-4.xlsx
@@ -1,48 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marvi\Desktop\Bachelor-Thesis\Testdaten\Testdaten von und für GPT-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE935546-DDCC-4654-9500-B932A74AE2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89FF092C-FB14-4068-878B-6837BBB3025F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarios" sheetId="1" r:id="rId1"/>
     <sheet name="Register" sheetId="2" r:id="rId2"/>
     <sheet name="Login" sheetId="3" r:id="rId3"/>
-    <sheet name="Forgot Password" sheetId="4" r:id="rId4"/>
-    <sheet name="Search" sheetId="5" r:id="rId5"/>
-    <sheet name="Product Display Page" sheetId="6" r:id="rId6"/>
-    <sheet name="Add to Cart" sheetId="7" r:id="rId7"/>
-    <sheet name="Wish List" sheetId="8" r:id="rId8"/>
-    <sheet name="Shopping Cart" sheetId="9" r:id="rId9"/>
-    <sheet name="Home Page" sheetId="10" r:id="rId10"/>
-    <sheet name="Checkout" sheetId="11" r:id="rId11"/>
-    <sheet name="My Account" sheetId="12" r:id="rId12"/>
-    <sheet name="My Account Information" sheetId="13" r:id="rId13"/>
-    <sheet name="Change Password" sheetId="14" r:id="rId14"/>
-    <sheet name="Address Book" sheetId="15" r:id="rId15"/>
-    <sheet name="Order History" sheetId="16" r:id="rId16"/>
-    <sheet name="Order Information" sheetId="17" r:id="rId17"/>
-    <sheet name="Product Returns" sheetId="18" r:id="rId18"/>
-    <sheet name="Downloads" sheetId="19" r:id="rId19"/>
-    <sheet name="Reward Points" sheetId="20" r:id="rId20"/>
-    <sheet name="Returns" sheetId="21" r:id="rId21"/>
-    <sheet name="Transactions" sheetId="22" r:id="rId22"/>
-    <sheet name="Recurring Payments" sheetId="23" r:id="rId23"/>
-    <sheet name="Affiliate" sheetId="24" r:id="rId24"/>
-    <sheet name="Newsletter" sheetId="25" r:id="rId25"/>
-    <sheet name="Contact Us" sheetId="26" r:id="rId26"/>
-    <sheet name="Gift Certificate" sheetId="27" r:id="rId27"/>
-    <sheet name="Specail Offers" sheetId="28" r:id="rId28"/>
-    <sheet name="Header Menu Footer Options" sheetId="29" r:id="rId29"/>
-    <sheet name="Currencies" sheetId="30" r:id="rId30"/>
+    <sheet name="Logout" sheetId="31" r:id="rId4"/>
+    <sheet name="Forgot Password" sheetId="4" r:id="rId5"/>
+    <sheet name="Search" sheetId="5" r:id="rId6"/>
+    <sheet name="Product Display Page" sheetId="6" r:id="rId7"/>
+    <sheet name="Add to Cart" sheetId="7" r:id="rId8"/>
+    <sheet name="Wish List" sheetId="8" r:id="rId9"/>
+    <sheet name="Shopping Cart" sheetId="9" r:id="rId10"/>
+    <sheet name="Home Page" sheetId="10" r:id="rId11"/>
+    <sheet name="Checkout" sheetId="11" r:id="rId12"/>
+    <sheet name="My Account" sheetId="12" r:id="rId13"/>
+    <sheet name="My Account Information" sheetId="13" r:id="rId14"/>
+    <sheet name="Change Password" sheetId="14" r:id="rId15"/>
+    <sheet name="Address Book" sheetId="15" r:id="rId16"/>
+    <sheet name="Order History" sheetId="16" r:id="rId17"/>
+    <sheet name="Order Information" sheetId="17" r:id="rId18"/>
+    <sheet name="Product Returns" sheetId="18" r:id="rId19"/>
+    <sheet name="Downloads" sheetId="19" r:id="rId20"/>
+    <sheet name="Reward Points" sheetId="20" r:id="rId21"/>
+    <sheet name="Returns" sheetId="21" r:id="rId22"/>
+    <sheet name="Transactions" sheetId="22" r:id="rId23"/>
+    <sheet name="Recurring Payments" sheetId="23" r:id="rId24"/>
+    <sheet name="Affiliate" sheetId="24" r:id="rId25"/>
+    <sheet name="Newsletter" sheetId="25" r:id="rId26"/>
+    <sheet name="Contact Us" sheetId="26" r:id="rId27"/>
+    <sheet name="Gift Certificate" sheetId="27" r:id="rId28"/>
+    <sheet name="Specail Offers" sheetId="28" r:id="rId29"/>
+    <sheet name="Header Menu Footer Options" sheetId="29" r:id="rId30"/>
+    <sheet name="Currencies" sheetId="30" r:id="rId31"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="244">
   <si>
     <t>Test Scenario Description</t>
   </si>
@@ -759,6 +760,123 @@
   </si>
   <si>
     <t>User is redirected to login page</t>
+  </si>
+  <si>
+    <t>Successful Logout</t>
+  </si>
+  <si>
+    <t>Open OpenCart.com, User is logged into OpenCart account</t>
+  </si>
+  <si>
+    <t>Valid Logout</t>
+  </si>
+  <si>
+    <t>1. Click on 'Logout' button</t>
+  </si>
+  <si>
+    <t>User is redirected to the homepage, Login/Register buttons are visible</t>
+  </si>
+  <si>
+    <t>Verify UI elements after Logout</t>
+  </si>
+  <si>
+    <t>UI Verification</t>
+  </si>
+  <si>
+    <t>1. Click on 'Logout' button
+2. Verify if 'Login' and 'Register' buttons appear in the navigation bar</t>
+  </si>
+  <si>
+    <t>Navigation elements should be updated, Account-related options should disappear</t>
+  </si>
+  <si>
+    <t>Logout and Attempt to Access Account Page</t>
+  </si>
+  <si>
+    <t>1. Click on 'Logout' button
+2. Try to access the 'Account' page directly</t>
+  </si>
+  <si>
+    <t>User is redirected to the login page</t>
+  </si>
+  <si>
+    <t>Logout and Browser Back Navigation</t>
+  </si>
+  <si>
+    <t>1. Click on 'Logout' button
+2. Press the browser 'Back' button</t>
+  </si>
+  <si>
+    <t>User should not be able to access the previous session, redirected to login page</t>
+  </si>
+  <si>
+    <t>Logout and Attempt to Access Secure Page via URL</t>
+  </si>
+  <si>
+    <t>1. Click on 'Logout' button
+2. Open a secure page (e.g., dashboard) via URL</t>
+  </si>
+  <si>
+    <t>Logout During Active Session on Another Page</t>
+  </si>
+  <si>
+    <t>Session Management</t>
+  </si>
+  <si>
+    <t>1. Navigate to another section (e.g., Purchases)
+2. Click on 'Logout' button</t>
+  </si>
+  <si>
+    <t>User is logged out across all active sessions</t>
+  </si>
+  <si>
+    <t>Automatic Logout After Inactivity</t>
+  </si>
+  <si>
+    <t>Timeout Scenario</t>
+  </si>
+  <si>
+    <t>1. Stay inactive for 30 minutes
+2. Try to perform any action</t>
+  </si>
+  <si>
+    <t>User is automatically logged out and redirected to the login page</t>
+  </si>
+  <si>
+    <t>Logout and Immediate Login Attempt</t>
+  </si>
+  <si>
+    <t>Login Verification</t>
+  </si>
+  <si>
+    <t>1. Click on 'Logout' button
+2. Click 'Login' and enter credentials</t>
+  </si>
+  <si>
+    <t>User should be able to log in again successfully</t>
+  </si>
+  <si>
+    <t>Verify Logout Button Visibility</t>
+  </si>
+  <si>
+    <t>1. Click on 'Logout' button
+2. Check if 'Logout' button disappears from the navigation bar</t>
+  </si>
+  <si>
+    <t>Logout and Refresh the Page</t>
+  </si>
+  <si>
+    <t>1. Click on 'Logout' button
+2. Refresh the browser page</t>
+  </si>
+  <si>
+    <t>User should remain logged out, Login/Register buttons remain visible</t>
+  </si>
+  <si>
+    <t>Logout' button should not be visible after logout</t>
+  </si>
+  <si>
+    <t>Test Scenario Descripton von Pavankumar21github [2022]</t>
   </si>
 </sst>
 </file>
@@ -851,7 +969,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -878,6 +996,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1171,22 +1292,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="74.28515625" customWidth="1"/>
     <col min="2" max="2" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="36" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="36" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1194,7 +1318,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1202,67 +1326,70 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="36" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" ht="36" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -1356,6 +1483,15 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69D18EF4-CB07-482B-8120-500AFEA41AAD}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F59ECDB-6887-412D-AE40-CAEFBBF69F30}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1364,7 +1500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E3281B2-ECE2-4229-8E21-DD0154D6B597}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1373,7 +1509,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC891B4D-CEB7-428C-AF11-DCFCD005A99F}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1382,7 +1518,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67FE3611-CBBC-427E-B012-E6C8579C6CA3}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1391,7 +1527,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74085656-08C1-43DA-983A-046601A87472}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1400,7 +1536,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{884EF907-734D-47C2-A462-0A7DDD7773AA}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1409,7 +1545,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8E5B671-0B83-466E-B4C9-A5B4C2F32FB0}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1418,7 +1554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAAF1EEB-08B3-4462-A935-285A740C21B1}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1427,17 +1563,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB318571-7AA6-48E7-8B34-1554E4D4D71F}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6366D9F1-B0C3-4E0E-A154-D57D8B3B5093}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1884,6 +2011,15 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6366D9F1-B0C3-4E0E-A154-D57D8B3B5093}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBD04566-2B9F-4B07-AA34-BF57464EB60D}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1892,7 +2028,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E879D26-DF42-416A-B355-648FF3505B03}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1901,7 +2037,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2166216-EEEF-4E1B-B517-FAF39C77E32F}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1910,7 +2046,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B3BDDD2-D55F-46D4-BF02-5AC4E8168912}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1919,7 +2055,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51240DEB-4720-4744-A3E5-ABE3B15218B8}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1928,7 +2064,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F321C8C-3303-4D7C-9741-9B98D2CB30B9}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1937,7 +2073,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D0881DA-FFFD-4EA2-A7CE-6EEFF29BDA2D}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1946,7 +2082,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C6C93B5-A0D8-4D55-82E6-2C662B74A26E}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1955,17 +2091,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62A08BA0-82AB-40C6-AB10-9C065EBEE794}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC3A216-5155-4CEF-8A20-6800539D6F36}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -2452,6 +2579,15 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC3A216-5155-4CEF-8A20-6800539D6F36}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83B7116B-4DF8-4BB1-9D76-F6F969D5F7C7}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2461,6 +2597,266 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{145866A2-7F89-4E13-BC2A-2C04982FBE24}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="6" max="6" width="20.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+    </row>
+    <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+    </row>
+    <row r="4" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+    </row>
+    <row r="6" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+    </row>
+    <row r="7" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+    </row>
+    <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+    </row>
+    <row r="10" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+    </row>
+    <row r="11" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B87FF5BC-0666-433A-9ADB-FC60B68CC696}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2469,7 +2865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACCF51F9-3319-459B-87DB-F023A541C9C3}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2478,7 +2874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF293EA0-B5E7-4CA4-88EA-BB5093B9A174}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2487,7 +2883,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8819886F-B11A-44ED-87B0-0DB3C124ED3B}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2496,20 +2892,11 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C77B75-3DB4-41BB-A87D-FCE0B7306371}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69D18EF4-CB07-482B-8120-500AFEA41AAD}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Quellenverzeichnis + Forgot Passwort
</commit_message>
<xml_diff>
--- a/Testdaten/Testdaten von und für GPT-4/OpenCart-TestExecution Results_GPT-4.xlsx
+++ b/Testdaten/Testdaten von und für GPT-4/OpenCart-TestExecution Results_GPT-4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marvi\Desktop\Bachelor-Thesis\Testdaten\Testdaten von und für GPT-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89FF092C-FB14-4068-878B-6837BBB3025F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A671A67F-8D0C-4E8D-B248-5B0ACACB2898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarios" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="318">
   <si>
     <t>Test Scenario Description</t>
   </si>
@@ -877,6 +877,259 @@
   </si>
   <si>
     <t>Test Scenario Descripton von Pavankumar21github [2022]</t>
+  </si>
+  <si>
+    <t>Request Password Reset with Valid Email</t>
+  </si>
+  <si>
+    <t>Open OpenCart.com, User is on the 'Forgot Password' page, An existing account is required</t>
+  </si>
+  <si>
+    <t>Valid Reset Request</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Enter a registered email
+3. Click 'Submit'</t>
+  </si>
+  <si>
+    <t>Success message: 'An email with a reset link has been sent'</t>
+  </si>
+  <si>
+    <t>Request Password Reset with Unregistered Email</t>
+  </si>
+  <si>
+    <t>Open OpenCart.com, User is on the 'Forgot Password' page</t>
+  </si>
+  <si>
+    <t>Invalid Reset Request</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Enter an unregistered email
+3. Click 'Submit'</t>
+  </si>
+  <si>
+    <t>Error message: 'E-Mail Address does not appear to be valid!'</t>
+  </si>
+  <si>
+    <t>Request Password Reset with Empty Email Field</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Leave the email field empty
+3. Click 'Submit'</t>
+  </si>
+  <si>
+    <t>Access Password Reset Link</t>
+  </si>
+  <si>
+    <t>Open OpenCart.com, User has received the password reset email, An existing account is required</t>
+  </si>
+  <si>
+    <t>Verify Reset Link</t>
+  </si>
+  <si>
+    <t>1. Click on the password reset link in the email</t>
+  </si>
+  <si>
+    <t>User is redirected to the 'Reset Password' page</t>
+  </si>
+  <si>
+    <t>Attempt to Use Expired Password Reset Link</t>
+  </si>
+  <si>
+    <t>Invalid Reset Link</t>
+  </si>
+  <si>
+    <t>1. Click on an expired reset link</t>
+  </si>
+  <si>
+    <t>Error message: 'The password reset link has expired!'</t>
+  </si>
+  <si>
+    <t>Reset Password with Matching New Passwords</t>
+  </si>
+  <si>
+    <t>Open OpenCart.com, User is on the 'Reset Password' page, User has received the password reset email, An existing account is required</t>
+  </si>
+  <si>
+    <t>Valid Password Reset</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Enter a new valid password
+3. Re-enter the same password
+4. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>Success message: 'Your password has been updated'</t>
+  </si>
+  <si>
+    <t>Reset Password with Non-Matching Confirmation</t>
+  </si>
+  <si>
+    <t>Invalid Password Reset</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Enter a new password
+3. Enter a different confirmation password
+4. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>Error message: 'Passwords do not match!'</t>
+  </si>
+  <si>
+    <t>Reset Password with Weak Password</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Enter a weak password (e.g., too short)
+3. Enter the same confirmation password
+4. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>Error message: 'Password does not meet security requirements!'</t>
+  </si>
+  <si>
+    <t>Reset Password with Empty Fields</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Leave both password fields empty
+3. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>Error message: 'Password fields cannot be empty!'</t>
+  </si>
+  <si>
+    <t>Login After Successful Password Reset</t>
+  </si>
+  <si>
+    <t>Verify New Password</t>
+  </si>
+  <si>
+    <t>1. Enter email and new password on the login page
+2. Click 'Login'</t>
+  </si>
+  <si>
+    <t>UI Verification of Password Reset Page</t>
+  </si>
+  <si>
+    <t>1. Verify presence of 'E-Mail Address' field
+2. Verify 'Submit' button is visible</t>
+  </si>
+  <si>
+    <t>All UI elements should be visible and functional</t>
+  </si>
+  <si>
+    <t>UI Verification of Reset Password Page</t>
+  </si>
+  <si>
+    <t>Open OpenCart.com, User is on the 'Reset Password' page, User has received the password reset email</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Verify presence of 'Password' and 'Confirm Password' fields
+3. Verify 'Continue' button is visible</t>
+  </si>
+  <si>
+    <t>Verify Navigation Back to Login Page</t>
+  </si>
+  <si>
+    <t>1. Click on 'Login?' link</t>
+  </si>
+  <si>
+    <t>Request Another Password Reset Without Waiting</t>
+  </si>
+  <si>
+    <t>Reset Request Spam Check</t>
+  </si>
+  <si>
+    <t>1. Enter a registered email
+2. Click 'Submit' twice in quick succession</t>
+  </si>
+  <si>
+    <t>Verify if multiple reset emails are sent or system blocks rapid requests</t>
+  </si>
+  <si>
+    <t>Verify Logout After Password Reset</t>
+  </si>
+  <si>
+    <t>1. Complete password reset
+2. Try to use old password to log in</t>
+  </si>
+  <si>
+    <t>Old password should no longer work</t>
+  </si>
+  <si>
+    <t>Attempt to Use Reset Link After Password Change</t>
+  </si>
+  <si>
+    <t>1. Change password successfully
+2. Try to use the old reset link</t>
+  </si>
+  <si>
+    <t>Reset Password and Attempt Old Password Login</t>
+  </si>
+  <si>
+    <t>1. Click on 'Forgotten Password' link from Login page
+2. Change password successfully
+3. Try to log in with the old password</t>
+  </si>
+  <si>
+    <t>Old password should not work, only new password is valid</t>
+  </si>
+  <si>
+    <t>Verify Reset Email Not Received Due to Incorrect Address</t>
+  </si>
+  <si>
+    <t>Email Delivery Check</t>
+  </si>
+  <si>
+    <t>1. Enter a wrongly formatted email
+2. Click 'Submit'</t>
+  </si>
+  <si>
+    <t>Verify Password Field Masking</t>
+  </si>
+  <si>
+    <t>1. Enter a password
+2. Verify characters are masked</t>
+  </si>
+  <si>
+    <t>Password input should be hidden behind dots or asterisks</t>
+  </si>
+  <si>
+    <t>Verify Special Characters Allowed in Password</t>
+  </si>
+  <si>
+    <t>Validation Check</t>
+  </si>
+  <si>
+    <t>1. Enter a password with special characters
+2. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>Password should be accepted if it meets security criteria</t>
+  </si>
+  <si>
+    <t>Verify Minimum Password Length Requirement</t>
+  </si>
+  <si>
+    <t>1. Enter a password shorter than the required length
+2. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>Verify Maximum Password Length Handling</t>
+  </si>
+  <si>
+    <t>1. Enter an extremely long password
+2. Click 'Continue'</t>
+  </si>
+  <si>
+    <t>Either an error is displayed, or the input is truncated</t>
   </si>
 </sst>
 </file>
@@ -969,7 +1222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1000,6 +1253,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1338,6 +1597,9 @@
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>22</v>
+      </c>
     </row>
     <row r="6" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -2858,9 +3120,524 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B87FF5BC-0666-433A-9ADB-FC60B68CC696}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+    </row>
+    <row r="2" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+    </row>
+    <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+    </row>
+    <row r="4" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+    </row>
+    <row r="5" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+    </row>
+    <row r="7" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+    </row>
+    <row r="9" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+    </row>
+    <row r="11" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+    </row>
+    <row r="12" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+    </row>
+    <row r="13" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+    </row>
+    <row r="14" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>292</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>299</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>301</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>304</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>305</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+    </row>
+    <row r="20" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+    </row>
+    <row r="21" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>311</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>312</v>
+      </c>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+    </row>
+    <row r="22" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>314</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+    </row>
+    <row r="23" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Tabellen + My Account Information Daten
</commit_message>
<xml_diff>
--- a/Testdaten/Testdaten von und für GPT-4/OpenCart-TestExecution Results_GPT-4.xlsx
+++ b/Testdaten/Testdaten von und für GPT-4/OpenCart-TestExecution Results_GPT-4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marvi\Desktop\Bachelor-Thesis\Testdaten\Testdaten von und für GPT-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74B66CD-3A97-4587-8FB4-142B36475E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDFA6B57-865B-4C28-9602-76D1E18A2957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,29 +19,25 @@
     <sheet name="Logout" sheetId="31" r:id="rId4"/>
     <sheet name="Forgot Password" sheetId="4" r:id="rId5"/>
     <sheet name="Add to Cart" sheetId="7" r:id="rId6"/>
-    <sheet name="Wish List" sheetId="8" r:id="rId7"/>
-    <sheet name="Shopping Cart" sheetId="9" r:id="rId8"/>
-    <sheet name="Home Page" sheetId="10" r:id="rId9"/>
-    <sheet name="Checkout" sheetId="11" r:id="rId10"/>
-    <sheet name="My Account" sheetId="12" r:id="rId11"/>
-    <sheet name="My Account Information" sheetId="13" r:id="rId12"/>
-    <sheet name="Change Password" sheetId="14" r:id="rId13"/>
-    <sheet name="Address Book" sheetId="15" r:id="rId14"/>
-    <sheet name="Order History" sheetId="16" r:id="rId15"/>
-    <sheet name="Order Information" sheetId="17" r:id="rId16"/>
-    <sheet name="Product Returns" sheetId="18" r:id="rId17"/>
-    <sheet name="Downloads" sheetId="19" r:id="rId18"/>
-    <sheet name="Reward Points" sheetId="20" r:id="rId19"/>
-    <sheet name="Returns" sheetId="21" r:id="rId20"/>
-    <sheet name="Transactions" sheetId="22" r:id="rId21"/>
-    <sheet name="Recurring Payments" sheetId="23" r:id="rId22"/>
-    <sheet name="Affiliate" sheetId="24" r:id="rId23"/>
-    <sheet name="Newsletter" sheetId="25" r:id="rId24"/>
-    <sheet name="Contact Us" sheetId="26" r:id="rId25"/>
-    <sheet name="Gift Certificate" sheetId="27" r:id="rId26"/>
-    <sheet name="Specail Offers" sheetId="28" r:id="rId27"/>
-    <sheet name="Header Menu Footer Options" sheetId="29" r:id="rId28"/>
-    <sheet name="Currencies" sheetId="30" r:id="rId29"/>
+    <sheet name="My Account" sheetId="12" r:id="rId7"/>
+    <sheet name="My Account Information" sheetId="13" r:id="rId8"/>
+    <sheet name="Change Password" sheetId="14" r:id="rId9"/>
+    <sheet name="Address Book" sheetId="15" r:id="rId10"/>
+    <sheet name="Order History" sheetId="16" r:id="rId11"/>
+    <sheet name="Order Information" sheetId="17" r:id="rId12"/>
+    <sheet name="Product Returns" sheetId="18" r:id="rId13"/>
+    <sheet name="Downloads" sheetId="19" r:id="rId14"/>
+    <sheet name="Reward Points" sheetId="20" r:id="rId15"/>
+    <sheet name="Returns" sheetId="21" r:id="rId16"/>
+    <sheet name="Transactions" sheetId="22" r:id="rId17"/>
+    <sheet name="Recurring Payments" sheetId="23" r:id="rId18"/>
+    <sheet name="Affiliate" sheetId="24" r:id="rId19"/>
+    <sheet name="Newsletter" sheetId="25" r:id="rId20"/>
+    <sheet name="Contact Us" sheetId="26" r:id="rId21"/>
+    <sheet name="Gift Certificate" sheetId="27" r:id="rId22"/>
+    <sheet name="Specail Offers" sheetId="28" r:id="rId23"/>
+    <sheet name="Header Menu Footer Options" sheetId="29" r:id="rId24"/>
+    <sheet name="Currencies" sheetId="30" r:id="rId25"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,19 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="355">
-  <si>
-    <t>Validate the working of 'Wish List' functionality</t>
-  </si>
-  <si>
-    <t>Validate the working of 'Shopping Cart' functionality</t>
-  </si>
-  <si>
-    <t>Validate the working of Home Page functionality</t>
-  </si>
-  <si>
-    <t>Verifty the working of Checkout functionality</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="388">
   <si>
     <t>Validate the My Account functionality</t>
   </si>
@@ -1273,6 +1257,130 @@
   </si>
   <si>
     <t>Test Szenario auf Open Car+A1:B14t</t>
+  </si>
+  <si>
+    <t>Modify Profile Picture</t>
+  </si>
+  <si>
+    <t>Verify Notification Preferences</t>
+  </si>
+  <si>
+    <t>Login to OpenCart</t>
+  </si>
+  <si>
+    <t>User Login</t>
+  </si>
+  <si>
+    <t>1. Click on 'Login' button
+2. Enter valid Email and Password
+3. Click 'Login' button</t>
+  </si>
+  <si>
+    <t>User is successfully logged in and redirected to the account page</t>
+  </si>
+  <si>
+    <t>Navigate to My Account</t>
+  </si>
+  <si>
+    <t>User is logged in</t>
+  </si>
+  <si>
+    <t>Account Navigation</t>
+  </si>
+  <si>
+    <t>1. Click on 'Account' button
+2. Click on 'Account Details'</t>
+  </si>
+  <si>
+    <t>User is navigated to the Account Details page</t>
+  </si>
+  <si>
+    <t>Verify Account Details Page</t>
+  </si>
+  <si>
+    <t>User is on Account Details page</t>
+  </si>
+  <si>
+    <t>1. Verify all fields are visible (Username, First Name, Last Name, Email, etc.)
+2. Verify Profile Picture section is visible
+3. Verify Submit and Cancel buttons are present</t>
+  </si>
+  <si>
+    <t>All elements are correctly displayed on the Account Details page</t>
+  </si>
+  <si>
+    <t>Update Account Information</t>
+  </si>
+  <si>
+    <t>Modify Account Data</t>
+  </si>
+  <si>
+    <t>1. Modify First Name and Last Name fields
+2. Click 'Submit' button</t>
+  </si>
+  <si>
+    <t>Success message: 'Your account details have been successfully updated!'</t>
+  </si>
+  <si>
+    <t>Verify Error for Duplicate Username</t>
+  </si>
+  <si>
+    <t>1. Enter an already registered username
+2. Click 'Submit' button</t>
+  </si>
+  <si>
+    <t>Error message: 'Username is already registered!'</t>
+  </si>
+  <si>
+    <t>Verify Error for Empty Required Fields</t>
+  </si>
+  <si>
+    <t>1. Clear First Name and Last Name fields
+2. Click 'Submit' button</t>
+  </si>
+  <si>
+    <t>Error message: 'First Name must be between 1 and 32 characters!'</t>
+  </si>
+  <si>
+    <t>Verify Profile Picture Upload</t>
+  </si>
+  <si>
+    <t>1. Click 'Browse' button under Profile Picture
+2. Select an image file
+3. Click 'Submit' button</t>
+  </si>
+  <si>
+    <t>Profile picture is successfully updated</t>
+  </si>
+  <si>
+    <t>Modify Preferences</t>
+  </si>
+  <si>
+    <t>1. Select 'Yes' for Notify Extension Updates
+2. Click 'Submit' button</t>
+  </si>
+  <si>
+    <t>Notification preference is successfully updated</t>
+  </si>
+  <si>
+    <t>Navigate via Dashboard</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>1. Click 'Dashboard' button
+2. Click 'Account Details'</t>
+  </si>
+  <si>
+    <t>Successful Account Update</t>
+  </si>
+  <si>
+    <t>Update Account Details</t>
+  </si>
+  <si>
+    <t>1. Modify any field with valid data
+2. Click 'Submit' button</t>
   </si>
 </sst>
 </file>
@@ -1443,8 +1551,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2D91B3ED-BFB3-4BF6-B9E2-B45047E3BC66}" name="Tabelle1" displayName="Tabelle1" ref="A1:B26" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
-  <autoFilter ref="A1:B26" xr:uid="{2D91B3ED-BFB3-4BF6-B9E2-B45047E3BC66}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2D91B3ED-BFB3-4BF6-B9E2-B45047E3BC66}" name="Tabelle1" displayName="Tabelle1" ref="A1:B22" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+  <autoFilter ref="A1:B22" xr:uid="{2D91B3ED-BFB3-4BF6-B9E2-B45047E3BC66}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{AFD0C039-7F58-456D-9118-3E6C37D5AFFD}" name="Test Szenario auf Open Car+A1:B14t" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{22051654-053C-48DC-A251-B2AACFF72BDF}" name="Number of Test Cases" dataDxfId="0"/>
@@ -1716,7 +1824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D279CBF0-E909-4C39-954E-02A0B1FE8668}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" customWidth="1"/>
@@ -1725,15 +1833,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="B2" s="2">
         <v>20</v>
@@ -1741,7 +1849,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B3" s="2">
         <v>22</v>
@@ -1749,7 +1857,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="B4" s="2">
         <v>10</v>
@@ -1757,7 +1865,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="B5" s="2">
         <v>22</v>
@@ -1765,7 +1873,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B6" s="2">
         <v>9</v>
@@ -1777,25 +1885,27 @@
       </c>
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B9" s="2"/>
     </row>
-    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>4</v>
       </c>
@@ -1843,53 +1953,29 @@
       </c>
       <c r="B18" s="2"/>
     </row>
-    <row r="19" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B19" s="2"/>
     </row>
-    <row r="20" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>13</v>
       </c>
       <c r="B20" s="2"/>
     </row>
-    <row r="21" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
+    <row r="21" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B21" s="2"/>
     </row>
-    <row r="22" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" s="2"/>
-    </row>
-    <row r="23" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B24" s="2"/>
-    </row>
-    <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B25" s="2"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
-        <v>353</v>
-      </c>
-      <c r="B26" s="2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="B22" s="2">
         <v>3</v>
       </c>
     </row>
@@ -1902,7 +1988,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E3281B2-ECE2-4229-8E21-DD0154D6B597}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{884EF907-734D-47C2-A462-0A7DDD7773AA}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1911,7 +1997,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC891B4D-CEB7-428C-AF11-DCFCD005A99F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8E5B671-0B83-466E-B4C9-A5B4C2F32FB0}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1920,7 +2006,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67FE3611-CBBC-427E-B012-E6C8579C6CA3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAAF1EEB-08B3-4462-A935-285A740C21B1}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1929,7 +2015,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74085656-08C1-43DA-983A-046601A87472}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB318571-7AA6-48E7-8B34-1554E4D4D71F}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1938,7 +2024,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{884EF907-734D-47C2-A462-0A7DDD7773AA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6366D9F1-B0C3-4E0E-A154-D57D8B3B5093}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1947,7 +2033,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8E5B671-0B83-466E-B4C9-A5B4C2F32FB0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBD04566-2B9F-4B07-AA34-BF57464EB60D}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1956,7 +2042,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAAF1EEB-08B3-4462-A935-285A740C21B1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E879D26-DF42-416A-B355-648FF3505B03}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1965,7 +2051,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB318571-7AA6-48E7-8B34-1554E4D4D71F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2166216-EEEF-4E1B-B517-FAF39C77E32F}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1974,7 +2060,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6366D9F1-B0C3-4E0E-A154-D57D8B3B5093}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B3BDDD2-D55F-46D4-BF02-5AC4E8168912}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1983,7 +2069,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBD04566-2B9F-4B07-AA34-BF57464EB60D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51240DEB-4720-4744-A3E5-ABE3B15218B8}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -2006,422 +2092,422 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2430,7 +2516,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E879D26-DF42-416A-B355-648FF3505B03}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F321C8C-3303-4D7C-9741-9B98D2CB30B9}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -2439,7 +2525,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2166216-EEEF-4E1B-B517-FAF39C77E32F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D0881DA-FFFD-4EA2-A7CE-6EEFF29BDA2D}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -2448,7 +2534,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B3BDDD2-D55F-46D4-BF02-5AC4E8168912}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C6C93B5-A0D8-4D55-82E6-2C662B74A26E}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -2457,7 +2543,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51240DEB-4720-4744-A3E5-ABE3B15218B8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62A08BA0-82AB-40C6-AB10-9C065EBEE794}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -2466,7 +2552,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F321C8C-3303-4D7C-9741-9B98D2CB30B9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC3A216-5155-4CEF-8A20-6800539D6F36}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -2475,42 +2561,6 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D0881DA-FFFD-4EA2-A7CE-6EEFF29BDA2D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C6C93B5-A0D8-4D55-82E6-2C662B74A26E}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62A08BA0-82AB-40C6-AB10-9C065EBEE794}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC3A216-5155-4CEF-8A20-6800539D6F36}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83B7116B-4DF8-4BB1-9D76-F6F969D5F7C7}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2525,82 +2575,82 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>21</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>344</v>
-      </c>
       <c r="F3" s="2" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -2623,462 +2673,462 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>141</v>
-      </c>
       <c r="F6" s="4" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D18" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>177</v>
-      </c>
       <c r="F18" s="4" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>186</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -3101,242 +3151,242 @@
   <sheetData>
     <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>195</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>199</v>
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E10" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>225</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>229</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
     </row>
     <row r="11" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -3361,506 +3411,506 @@
   <sheetData>
     <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>25</v>
       </c>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
     </row>
     <row r="2" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F2" s="7" t="s">
         <v>230</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>231</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>234</v>
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
     </row>
     <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>235</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>238</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>239</v>
       </c>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D4" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>241</v>
-      </c>
       <c r="F4" s="7" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>246</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
     </row>
     <row r="6" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
     </row>
     <row r="7" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>251</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>253</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>255</v>
       </c>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" ht="135" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D9" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>261</v>
-      </c>
       <c r="F9" s="7" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8" ht="135" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
     </row>
     <row r="17" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
     </row>
     <row r="18" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
     </row>
     <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
     </row>
     <row r="20" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
     </row>
     <row r="21" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
     </row>
     <row r="22" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D22" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="E22" s="7" t="s">
         <v>296</v>
       </c>
-      <c r="E22" s="7" t="s">
-        <v>300</v>
-      </c>
       <c r="F22" s="7" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
     </row>
     <row r="23" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
@@ -3885,202 +3935,202 @@
   <sheetData>
     <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="F2" s="7" t="s">
         <v>304</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>305</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="165" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D4" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>310</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D7" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>324</v>
-      </c>
       <c r="F7" s="7" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -4089,25 +4139,313 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C77B75-3DB4-41BB-A87D-FCE0B7306371}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC891B4D-CEB7-428C-AF11-DCFCD005A99F}">
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="17.140625" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69D18EF4-CB07-482B-8120-500AFEA41AAD}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67FE3611-CBBC-427E-B012-E6C8579C6CA3}">
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F59ECDB-6887-412D-AE40-CAEFBBF69F30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74085656-08C1-43DA-983A-046601A87472}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>